<commit_message>
feat: hapus 5 chart dashboard, tambah alamat warga & excel, perkuat keamanan sesi
</commit_message>
<xml_diff>
--- a/public/template_data_warga.xlsx
+++ b/public/template_data_warga.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:M3"/>
+  <dimension ref="A1:N3"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -434,9 +434,12 @@
         <v>Pekerjaan</v>
       </c>
       <c r="L1" t="str">
+        <v>Alamat</v>
+      </c>
+      <c r="M1" t="str">
         <v>No KK</v>
       </c>
-      <c r="M1" t="str">
+      <c r="N1" t="str">
         <v>Hubungan Keluarga</v>
       </c>
     </row>
@@ -475,9 +478,12 @@
         <v>Wiraswasta</v>
       </c>
       <c r="L2" t="str">
+        <v>Jl. Merdeka No. 10, RT 01 RW 02</v>
+      </c>
+      <c r="M2" t="str">
         <v>9876543210987654</v>
       </c>
-      <c r="M2" t="str">
+      <c r="N2" t="str">
         <v>Kepala Keluarga</v>
       </c>
     </row>
@@ -516,15 +522,18 @@
         <v>Ibu Rumah Tangga</v>
       </c>
       <c r="L3" t="str">
+        <v>Jl. Merdeka No. 10, RT 01 RW 02</v>
+      </c>
+      <c r="M3" t="str">
         <v>9876543210987654</v>
       </c>
-      <c r="M3" t="str">
+      <c r="N3" t="str">
         <v>Istri</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:M3"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:N3"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>